<commit_message>
May 19, 2026, 8:59 PM
</commit_message>
<xml_diff>
--- a/storage/exports/4/07TCRPS8655B1ZK/032026/gstr1.xlsx
+++ b/storage/exports/4/07TCRPS8655B1ZK/032026/gstr1.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="123">
   <si>
     <t>Summary For B2B, SEZ, DE (4A, 4B, 6B, 6C)</t>
   </si>
@@ -106,9 +106,6 @@
     <t>05-Uttarakhand</t>
   </si>
   <si>
-    <t>06-Haryana</t>
-  </si>
-  <si>
     <t>08-Rajasthan</t>
   </si>
   <si>
@@ -340,9 +337,6 @@
     <t>IN-7</t>
   </si>
   <si>
-    <t>LWABOG7260000001</t>
-  </si>
-  <si>
     <t>255724174047155204_1</t>
   </si>
   <si>
@@ -358,46 +352,37 @@
     <t>CANQ1W2600000013</t>
   </si>
   <si>
+    <t>CN-2</t>
+  </si>
+  <si>
+    <t>MFABNVY260000001</t>
+  </si>
+  <si>
+    <t>DAL84U2600000005</t>
+  </si>
+  <si>
+    <t>Sr. No. To</t>
+  </si>
+  <si>
+    <t>6p5kc26244</t>
+  </si>
+  <si>
+    <t>LWABOG7260000005</t>
+  </si>
+  <si>
+    <t>IN-9</t>
+  </si>
+  <si>
+    <t>6p5kc26C98</t>
+  </si>
+  <si>
     <t>LYAA9U7260000001</t>
   </si>
   <si>
-    <t>MFABNVY260000001</t>
-  </si>
-  <si>
-    <t>RAT6SO2600000028</t>
-  </si>
-  <si>
-    <t>DAL84U2600000005</t>
+    <t>RAT6SO2600000034</t>
   </si>
   <si>
     <t>LZAA9B7260000001</t>
-  </si>
-  <si>
-    <t>Sr. No. To</t>
-  </si>
-  <si>
-    <t>6p5kc26244</t>
-  </si>
-  <si>
-    <t>FAWRLX2600000107</t>
-  </si>
-  <si>
-    <t>IN-9</t>
-  </si>
-  <si>
-    <t>LWABOG7260000005</t>
-  </si>
-  <si>
-    <t>6p5kc26C98</t>
-  </si>
-  <si>
-    <t>CANQ1W2600000019</t>
-  </si>
-  <si>
-    <t>MFABNVY260000002</t>
-  </si>
-  <si>
-    <t>RAT6SO2600000034</t>
   </si>
   <si>
     <t>Total Number</t>
@@ -831,12 +816,12 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E1" t="s">
         <v>17</v>
@@ -844,15 +829,15 @@
     </row>
     <row r="2" spans="1:5">
       <c r="D2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="E2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="D3">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -860,30 +845,30 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C4" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D4" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="E4" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D5">
         <v>112</v>
@@ -894,16 +879,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C6" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D6">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -911,13 +896,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -928,13 +913,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C8" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D8">
         <v>3</v>
@@ -948,13 +933,13 @@
         <v>97</v>
       </c>
       <c r="B9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="D9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -962,13 +947,13 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -979,13 +964,13 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -996,16 +981,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -1013,16 +998,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C13" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D13">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -1030,16 +1015,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C14" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="D14">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -1047,16 +1032,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C15" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -1067,66 +1052,15 @@
         <v>98</v>
       </c>
       <c r="B16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C16" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D16">
         <v>2</v>
       </c>
       <c r="E16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" t="s">
-        <v>98</v>
-      </c>
-      <c r="B17" t="s">
-        <v>113</v>
-      </c>
-      <c r="C17" t="s">
-        <v>124</v>
-      </c>
-      <c r="D17">
-        <v>7</v>
-      </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" t="s">
-        <v>99</v>
-      </c>
-      <c r="B18" t="s">
-        <v>114</v>
-      </c>
-      <c r="C18" t="s">
-        <v>114</v>
-      </c>
-      <c r="D18">
-        <v>1</v>
-      </c>
-      <c r="E18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" t="s">
-        <v>99</v>
-      </c>
-      <c r="B19" t="s">
-        <v>115</v>
-      </c>
-      <c r="C19" t="s">
-        <v>115</v>
-      </c>
-      <c r="D19">
-        <v>1</v>
-      </c>
-      <c r="E19">
         <v>0</v>
       </c>
     </row>
@@ -1200,7 +1134,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1213,7 +1147,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="E2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F2" t="s">
         <v>18</v>
@@ -1221,7 +1155,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="E3">
-        <v>16681.17</v>
+        <v>16577.99</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -1312,7 +1246,7 @@
         <v>3</v>
       </c>
       <c r="E8">
-        <v>193.2</v>
+        <v>312.63</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -1329,7 +1263,7 @@
         <v>3</v>
       </c>
       <c r="E9">
-        <v>312.63</v>
+        <v>2211.99</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -1346,7 +1280,7 @@
         <v>3</v>
       </c>
       <c r="E10">
-        <v>2205.47</v>
+        <v>721.37</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -1363,7 +1297,7 @@
         <v>3</v>
       </c>
       <c r="E11">
-        <v>721.37</v>
+        <v>303.88</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -1380,7 +1314,7 @@
         <v>3</v>
       </c>
       <c r="E12">
-        <v>303.88</v>
+        <v>1062.14</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -1397,7 +1331,7 @@
         <v>3</v>
       </c>
       <c r="E13">
-        <v>1062.14</v>
+        <v>1320.38</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -1414,7 +1348,7 @@
         <v>3</v>
       </c>
       <c r="E14">
-        <v>1304.84</v>
+        <v>691.27</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -1431,7 +1365,7 @@
         <v>3</v>
       </c>
       <c r="E15">
-        <v>691.27</v>
+        <v>417.48</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -1448,7 +1382,7 @@
         <v>3</v>
       </c>
       <c r="E16">
-        <v>401.94</v>
+        <v>436.89</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -1465,7 +1399,7 @@
         <v>3</v>
       </c>
       <c r="E17">
-        <v>436.89</v>
+        <v>544.65</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1482,7 +1416,7 @@
         <v>3</v>
       </c>
       <c r="E18">
-        <v>538.83</v>
+        <v>1549.52</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -1499,7 +1433,7 @@
         <v>3</v>
       </c>
       <c r="E19">
-        <v>1549.52</v>
+        <v>1127.18</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -1516,7 +1450,7 @@
         <v>3</v>
       </c>
       <c r="E20">
-        <v>1127.18</v>
+        <v>1889.32</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -1533,7 +1467,7 @@
         <v>3</v>
       </c>
       <c r="E21">
-        <v>1842.72</v>
+        <v>1178.63</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -1550,7 +1484,7 @@
         <v>3</v>
       </c>
       <c r="E22">
-        <v>1178.63</v>
+        <v>1306.77</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -1567,26 +1501,9 @@
         <v>3</v>
       </c>
       <c r="E23">
-        <v>1306.77</v>
+        <v>679.61</v>
       </c>
       <c r="F23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24" t="s">
-        <v>43</v>
-      </c>
-      <c r="D24">
-        <v>3</v>
-      </c>
-      <c r="E24">
-        <v>679.61</v>
-      </c>
-      <c r="F24">
         <v>0</v>
       </c>
     </row>
@@ -1602,7 +1519,7 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="M1" t="s">
         <v>17</v>
@@ -1613,10 +1530,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L2" t="s">
         <v>15</v>
@@ -1650,13 +1567,13 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" t="s">
         <v>47</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>48</v>
-      </c>
-      <c r="E4" t="s">
-        <v>49</v>
       </c>
       <c r="F4" t="s">
         <v>9</v>
@@ -1665,10 +1582,10 @@
         <v>10</v>
       </c>
       <c r="H4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J4" t="s">
         <v>11</v>
@@ -1695,7 +1612,7 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K1" t="s">
         <v>17</v>
@@ -1703,22 +1620,22 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G2" t="s">
         <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K2" t="s">
         <v>18</v>
@@ -1749,19 +1666,19 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" t="s">
         <v>55</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>56</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>57</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>58</v>
-      </c>
-      <c r="E4" t="s">
-        <v>59</v>
       </c>
       <c r="F4" t="s">
         <v>14</v>
@@ -1770,13 +1687,13 @@
         <v>16</v>
       </c>
       <c r="H4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K4" t="s">
         <v>19</v>
@@ -1794,7 +1711,7 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K1" t="s">
         <v>17</v>
@@ -1802,22 +1719,22 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G2" t="s">
         <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K2" t="s">
         <v>18</v>
@@ -1848,19 +1765,19 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" t="s">
         <v>55</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>56</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>57</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>58</v>
-      </c>
-      <c r="E4" t="s">
-        <v>59</v>
       </c>
       <c r="F4" t="s">
         <v>14</v>
@@ -1869,13 +1786,13 @@
         <v>16</v>
       </c>
       <c r="H4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K4" t="s">
         <v>19</v>
@@ -1893,7 +1810,7 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K1" t="s">
         <v>17</v>
@@ -1901,22 +1818,22 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G2" t="s">
         <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K2" t="s">
         <v>18</v>
@@ -1947,19 +1864,19 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" t="s">
         <v>55</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>56</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>57</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>58</v>
-      </c>
-      <c r="E4" t="s">
-        <v>59</v>
       </c>
       <c r="F4" t="s">
         <v>14</v>
@@ -1968,13 +1885,13 @@
         <v>16</v>
       </c>
       <c r="H4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K4" t="s">
         <v>19</v>
@@ -1992,7 +1909,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D1" t="s">
         <v>17</v>
@@ -2000,13 +1917,13 @@
     </row>
     <row r="2" spans="1:4">
       <c r="B2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2022,36 +1939,36 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2066,7 +1983,7 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H1" t="s">
         <v>17</v>
@@ -2074,19 +1991,19 @@
     </row>
     <row r="2" spans="1:8">
       <c r="B2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H2" t="s">
         <v>18</v>
@@ -2097,10 +2014,10 @@
         <v>3</v>
       </c>
       <c r="D3">
-        <v>16681.17</v>
+        <v>16577.99</v>
       </c>
       <c r="E3">
-        <v>480.09</v>
+        <v>476.99</v>
       </c>
       <c r="F3">
         <v>10.21</v>
@@ -2114,45 +2031,45 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" t="s">
         <v>90</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>91</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>92</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>93</v>
-      </c>
-      <c r="H4" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D5">
-        <v>2563.71</v>
+        <v>2653.73</v>
       </c>
       <c r="E5">
-        <v>73.95999999999999</v>
+        <v>76.66</v>
       </c>
       <c r="F5">
         <v>1.5</v>
@@ -2166,19 +2083,19 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D6">
-        <v>1168.91</v>
+        <v>975.71</v>
       </c>
       <c r="E6">
-        <v>35.09</v>
+        <v>29.29</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -2192,13 +2109,13 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D7">
         <v>12948.55</v>

</xml_diff>

<commit_message>
May 19, 2026, 9:05 PM
</commit_message>
<xml_diff>
--- a/storage/exports/4/07TCRPS8655B1ZK/032026/gstr1.xlsx
+++ b/storage/exports/4/07TCRPS8655B1ZK/032026/gstr1.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="128">
   <si>
     <t>Summary For B2B, SEZ, DE (4A, 4B, 6B, 6C)</t>
   </si>
@@ -337,6 +337,9 @@
     <t>IN-7</t>
   </si>
   <si>
+    <t>LWABOG7260000001</t>
+  </si>
+  <si>
     <t>255724174047155204_1</t>
   </si>
   <si>
@@ -355,34 +358,46 @@
     <t>CN-2</t>
   </si>
   <si>
+    <t>LYAA9U7260000001</t>
+  </si>
+  <si>
     <t>MFABNVY260000001</t>
   </si>
   <si>
+    <t>RAT6SO2600000028</t>
+  </si>
+  <si>
     <t>DAL84U2600000005</t>
   </si>
   <si>
+    <t>LZAA9B7260000001</t>
+  </si>
+  <si>
     <t>Sr. No. To</t>
   </si>
   <si>
     <t>6p5kc26244</t>
   </si>
   <si>
+    <t>FAWRLX2600000107</t>
+  </si>
+  <si>
+    <t>IN-9</t>
+  </si>
+  <si>
     <t>LWABOG7260000005</t>
   </si>
   <si>
-    <t>IN-9</t>
-  </si>
-  <si>
     <t>6p5kc26C98</t>
   </si>
   <si>
-    <t>LYAA9U7260000001</t>
+    <t>CANQ1W2600000019</t>
+  </si>
+  <si>
+    <t>MFABNVY260000002</t>
   </si>
   <si>
     <t>RAT6SO2600000034</t>
-  </si>
-  <si>
-    <t>LZAA9B7260000001</t>
   </si>
   <si>
     <t>Total Number</t>
@@ -816,7 +831,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -829,10 +844,10 @@
     </row>
     <row r="2" spans="1:5">
       <c r="D2" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="E2" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -851,13 +866,13 @@
         <v>99</v>
       </c>
       <c r="C4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D4" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="E4" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -868,7 +883,7 @@
         <v>100</v>
       </c>
       <c r="C5" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D5">
         <v>112</v>
@@ -885,10 +900,10 @@
         <v>101</v>
       </c>
       <c r="C6" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D6">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -919,7 +934,7 @@
         <v>103</v>
       </c>
       <c r="C8" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D8">
         <v>3</v>
@@ -930,16 +945,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B9" t="s">
         <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -987,10 +1002,10 @@
         <v>107</v>
       </c>
       <c r="C12" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="D12">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -1004,10 +1019,10 @@
         <v>108</v>
       </c>
       <c r="C13" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D13">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -1021,10 +1036,10 @@
         <v>109</v>
       </c>
       <c r="C14" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="D14">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -1038,10 +1053,10 @@
         <v>110</v>
       </c>
       <c r="C15" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="D15">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -1049,18 +1064,86 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B16" t="s">
         <v>111</v>
       </c>
       <c r="C16" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" t="s">
+        <v>112</v>
+      </c>
+      <c r="C17" t="s">
+        <v>123</v>
+      </c>
+      <c r="D17">
         <v>2</v>
       </c>
-      <c r="E16">
+      <c r="E17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>97</v>
+      </c>
+      <c r="B18" t="s">
+        <v>113</v>
+      </c>
+      <c r="C18" t="s">
+        <v>124</v>
+      </c>
+      <c r="D18">
+        <v>7</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B19" t="s">
+        <v>114</v>
+      </c>
+      <c r="C19" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>98</v>
+      </c>
+      <c r="B20" t="s">
+        <v>115</v>
+      </c>
+      <c r="C20" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
         <v>0</v>
       </c>
     </row>

</xml_diff>